<commit_message>
Consultas al servidor con reintentos y registro de promociones en el pedido
</commit_message>
<xml_diff>
--- a/excel/usuarios_funcionalidades.xlsx
+++ b/excel/usuarios_funcionalidades.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Usuarios!$A$1:$G$446</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -19,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="852">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="853">
   <si>
     <t>clave</t>
   </si>
@@ -2575,6 +2578,9 @@
   </si>
   <si>
     <t>EL POCHOLO FERRETERI</t>
+  </si>
+  <si>
+    <t>FERRIYAN 2 FERRETERI</t>
   </si>
 </sst>
 </file>
@@ -2895,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G446"/>
+  <dimension ref="A1:G447"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -9152,7 +9158,22 @@
         <v>10</v>
       </c>
     </row>
+    <row r="447" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A447">
+        <v>61001</v>
+      </c>
+      <c r="B447" t="s">
+        <v>852</v>
+      </c>
+      <c r="C447">
+        <v>61001</v>
+      </c>
+      <c r="E447" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:G446"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>